<commit_message>
ly: add stable PMC evidence locators
</commit_message>
<xml_diff>
--- a/data/interim/pmc_oa_candidate_pool_ly_v2_blind_annotation_v1_2026-10-03.xlsx
+++ b/data/interim/pmc_oa_candidate_pool_ly_v2_blind_annotation_v1_2026-10-03.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="1" r:id="Rc5f1ef713e7746ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blind_Annotation" sheetId="2" r:id="Re711cd1962e44f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="1" r:id="Re94f194a0fe14123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blind_Annotation" sheetId="2" r:id="Re24ee4d5ddec4c96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,14 +182,14 @@
   <x:dxfs count="4">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -199,7 +199,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -209,7 +209,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1013,7 +1013,7 @@
         <x:v>B0E94E71DA1EF955F0404E56EA4584E885A5A462D50FF0C6D9978C3BBFD7EB45</x:v>
       </x:c>
       <x:c r="U5" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC10715499; section=ABSTRACT; passage_index=2, offset=137; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC10715499/unicode</x:v>
       </x:c>
       <x:c r="V5" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1098,7 +1098,7 @@
         <x:v>B0E94E71DA1EF955F0404E56EA4584E885A5A462D50FF0C6D9978C3BBFD7EB45</x:v>
       </x:c>
       <x:c r="U6" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC10715499; section=ABSTRACT; passage_index=2, offset=137; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC10715499/unicode</x:v>
       </x:c>
       <x:c r="V6" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1183,7 +1183,7 @@
         <x:v>5F7B9C7EE6800A4235A04E84E0E66FF20C880F9970A58539D16B008E5C49D188</x:v>
       </x:c>
       <x:c r="U7" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC5007409; section=ABSTRACT; passage_index=2, offset=135; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC5007409/unicode</x:v>
       </x:c>
       <x:c r="V7" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1268,7 +1268,7 @@
         <x:v>9B1D983A7A23A645D10E51D25705BCBFC1AF0DDD0175CB2E2E5C6E051A36970E</x:v>
       </x:c>
       <x:c r="U8" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC10850450; section=ABSTRACT; passage_index=1, offset=96; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC10850450/unicode</x:v>
       </x:c>
       <x:c r="V8" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1353,7 +1353,7 @@
         <x:v>F05BAB6AE59FCB83879D3252F09BFD99128965BB38E674984F9F220EBA061A17</x:v>
       </x:c>
       <x:c r="U9" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC11309924; section=ABSTRACT; passage_index=2, offset=88; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC11309924/unicode</x:v>
       </x:c>
       <x:c r="V9" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1438,7 +1438,7 @@
         <x:v>3AF14372E644E6AC0FBB5F5E31F184E621E57D5DA3AE4BCA3F959BC4907BFF4F</x:v>
       </x:c>
       <x:c r="U10" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC12491465; section=ABSTRACT; passage_index=1, offset=103; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC12491465/unicode</x:v>
       </x:c>
       <x:c r="V10" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1523,7 +1523,7 @@
         <x:v>3224042ADA327689A9E94BEFC3A4A9D72DC2641C16640C51742869013113759F</x:v>
       </x:c>
       <x:c r="U11" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC6709302; section=ABSTRACT; passage_index=3, offset=68; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC6709302/unicode</x:v>
       </x:c>
       <x:c r="V11" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1608,7 +1608,7 @@
         <x:v>3224042ADA327689A9E94BEFC3A4A9D72DC2641C16640C51742869013113759F</x:v>
       </x:c>
       <x:c r="U12" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC6709302; section=ABSTRACT; passage_index=3, offset=68; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC6709302/unicode</x:v>
       </x:c>
       <x:c r="V12" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1693,7 +1693,7 @@
         <x:v>02088182D21EF32005CD48721432372EA163EC933A4F192BD96816F8170224BC</x:v>
       </x:c>
       <x:c r="U13" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC11984007; section=ABSTRACT; passage_index=2, offset=157; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC11984007/unicode</x:v>
       </x:c>
       <x:c r="V13" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1778,7 +1778,7 @@
         <x:v>86362B03404A617A45191ED3CC8667D7573FABDD3CA1EBA95DA2BCF7D5421ACE</x:v>
       </x:c>
       <x:c r="U14" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC7696452; section=ABSTRACT; passage_index=1, offset=119; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC7696452/unicode</x:v>
       </x:c>
       <x:c r="V14" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1863,7 +1863,7 @@
         <x:v>258F4875A40BC81DB5857056953F6246BF9162533993E7F50B93447314D14429</x:v>
       </x:c>
       <x:c r="U15" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC8793832; section=ABSTRACT; passage_index=1, offset=54; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC8793832/unicode</x:v>
       </x:c>
       <x:c r="V15" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -1948,7 +1948,7 @@
         <x:v>02BFF1BDD73534318E0FBC35D136525253C15F8EF1AEE51702AF01FED1BA5DD8</x:v>
       </x:c>
       <x:c r="U16" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC6982324; section=ABSTRACT; passage_index=1, offset=76; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC6982324/unicode</x:v>
       </x:c>
       <x:c r="V16" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2033,7 +2033,7 @@
         <x:v>02BFF1BDD73534318E0FBC35D136525253C15F8EF1AEE51702AF01FED1BA5DD8</x:v>
       </x:c>
       <x:c r="U17" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC6982324; section=ABSTRACT; passage_index=1, offset=76; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC6982324/unicode</x:v>
       </x:c>
       <x:c r="V17" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2118,7 +2118,7 @@
         <x:v>5FD3C8C7F06D6D14BD2C49669280BEBA191003E7ED69DC6E19D3758CA173A565</x:v>
       </x:c>
       <x:c r="U18" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC12297025; section=ABSTRACT; passage_index=1, offset=113; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC12297025/unicode</x:v>
       </x:c>
       <x:c r="V18" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2203,7 +2203,7 @@
         <x:v>E15FEB3B9C1F214896A9C03EC34708809F3C157C9AACC721973DB4D296BC0BEE</x:v>
       </x:c>
       <x:c r="U19" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC5839013; section=ABSTRACT; passage_index=2, offset=106; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC5839013/unicode</x:v>
       </x:c>
       <x:c r="V19" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2288,7 +2288,7 @@
         <x:v>21248D3DC1A802C26BD8409E281DE36313F756E9066F5995390A3BDDB668759D</x:v>
       </x:c>
       <x:c r="U20" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC7777221; section=ABSTRACT; passage_index=1, offset=92; passage_index=12, offset=2572; normalized evidence span (source punctuation/spacing differs); URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC7777221/unicode</x:v>
       </x:c>
       <x:c r="V20" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2373,7 +2373,7 @@
         <x:v>0D9956900CF18BD2E3A5989ADEDCB64DF8CA6072F835E69E1CC76C498841B489</x:v>
       </x:c>
       <x:c r="U21" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC9099525; section=ABSTRACT; passage_index=1, offset=120; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC9099525/unicode</x:v>
       </x:c>
       <x:c r="V21" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2458,7 +2458,7 @@
         <x:v>0D9956900CF18BD2E3A5989ADEDCB64DF8CA6072F835E69E1CC76C498841B489</x:v>
       </x:c>
       <x:c r="U22" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC9099525; section=ABSTRACT; passage_index=1, offset=120; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC9099525/unicode</x:v>
       </x:c>
       <x:c r="V22" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2543,7 +2543,7 @@
         <x:v>D8A58212983DA584C443227CDA58E433C5641F0D2AC81CBFF310AED1AA85D25D</x:v>
       </x:c>
       <x:c r="U23" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC6837311; section=ABSTRACT; passage_index=1, offset=80; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC6837311/unicode</x:v>
       </x:c>
       <x:c r="V23" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2628,7 +2628,7 @@
         <x:v>297804172E527105EE940E02A952E49FCBAA7821F97C7A80CF577F9B88D3497A</x:v>
       </x:c>
       <x:c r="U24" s="27" t="str">
-        <x:v>PMC full-text XML abstract paragraph 1; manual PDF page locator pending</x:v>
+        <x:v>NCBI PMC OA BioC JSON; PMC11177495; section=ABSTRACT; passage_index=1, offset=85; exact raw/normalized evidence passage; URL=https://www.ncbi.nlm.nih.gov/research/bionlp/RESTful/pmcoa.cgi/PMC11177495/unicode</x:v>
       </x:c>
       <x:c r="V24" s="27" t="str">
         <x:v>待与完整 train/dev/test、调参和评测清单复核</x:v>
@@ -2682,7 +2682,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25f22a6b77f24766"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R152904de908d47ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>